<commit_message>
visualize how often different actions are proposed (overall, by region, and by plan type)
</commit_message>
<xml_diff>
--- a/analysis/analyze_actions/action_evidence_coded.xlsx
+++ b/analysis/analyze_actions/action_evidence_coded.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/waana001/R Projects New/plan-analysis/analysis/analyze_actions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69A9B2CB-5EB8-8042-B293-D7B136C52327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43123509-58F1-B144-9216-E0F37FAC5DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{A32EED97-1107-FC45-88E1-AC5DB0786F2C}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="234">
   <si>
     <t>juris</t>
   </si>
@@ -542,9 +542,6 @@
     <t>assisted migration</t>
   </si>
   <si>
-    <t>climate refugia, connectivity</t>
-  </si>
-  <si>
     <t>connectivity</t>
   </si>
   <si>
@@ -677,9 +674,6 @@
     <t>connectivity; climate refugia</t>
   </si>
   <si>
-    <t>unclear (species selection and/or assisted migration)</t>
-  </si>
-  <si>
     <t>species selection; assisted migration</t>
   </si>
   <si>
@@ -725,7 +719,10 @@
     <t>South Central</t>
   </si>
   <si>
-    <t>USVI</t>
+    <t>coded based on context within plan</t>
+  </si>
+  <si>
+    <t>VI</t>
   </si>
 </sst>
 </file>
@@ -1636,13 +1633,13 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>192</v>
-      </c>
       <c r="C1" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>0</v>
@@ -1651,21 +1648,21 @@
         <v>1</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B2" s="5">
         <v>2025</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>2</v>
@@ -1680,13 +1677,13 @@
     </row>
     <row r="3" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B3" s="5">
         <v>2015</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>4</v>
@@ -1695,19 +1692,19 @@
         <v>5</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B4" s="5">
         <v>2025</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>6</v>
@@ -1716,19 +1713,19 @@
         <v>7</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G4" s="3"/>
     </row>
     <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B5" s="5">
         <v>2022</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>8</v>
@@ -1743,13 +1740,13 @@
     </row>
     <row r="6" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B6" s="5">
         <v>2022</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>8</v>
@@ -1758,19 +1755,19 @@
         <v>10</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B7" s="5">
         <v>2025</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>11</v>
@@ -1779,19 +1776,19 @@
         <v>12</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G7" s="3"/>
     </row>
     <row r="8" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B8" s="5">
         <v>2025</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>11</v>
@@ -1800,19 +1797,19 @@
         <v>13</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G8" s="3"/>
     </row>
     <row r="9" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B9" s="5">
         <v>2025</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>14</v>
@@ -1821,19 +1818,19 @@
         <v>15</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G9" s="3"/>
     </row>
     <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B10" s="5">
         <v>2025</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>14</v>
@@ -1842,19 +1839,19 @@
         <v>16</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G10" s="3"/>
     </row>
     <row r="11" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B11" s="5">
         <v>2015</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>17</v>
@@ -1863,19 +1860,19 @@
         <v>18</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G11" s="3"/>
     </row>
     <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B12" s="5">
         <v>2025</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>19</v>
@@ -1884,19 +1881,19 @@
         <v>20</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G12" s="3"/>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B13" s="5">
         <v>2025</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>19</v>
@@ -1911,13 +1908,13 @@
     </row>
     <row r="14" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B14" s="5">
         <v>2015</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>22</v>
@@ -1926,19 +1923,19 @@
         <v>23</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G14" s="3"/>
     </row>
     <row r="15" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B15" s="5">
         <v>2015</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>24</v>
@@ -1953,13 +1950,13 @@
     </row>
     <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B16" s="5">
         <v>2019</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>26</v>
@@ -1968,19 +1965,19 @@
         <v>27</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G16" s="3"/>
     </row>
     <row r="17" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B17" s="5">
         <v>2019</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>26</v>
@@ -1995,13 +1992,13 @@
     </row>
     <row r="18" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B18" s="5">
         <v>2015</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>29</v>
@@ -2016,13 +2013,13 @@
     </row>
     <row r="19" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B19" s="5">
         <v>2025</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>31</v>
@@ -2037,13 +2034,13 @@
     </row>
     <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B20" s="5">
         <v>2025</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>31</v>
@@ -2058,13 +2055,13 @@
     </row>
     <row r="21" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B21" s="5">
         <v>2023</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>34</v>
@@ -2073,19 +2070,19 @@
         <v>35</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G21" s="3"/>
     </row>
     <row r="22" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B22" s="5">
         <v>2023</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>34</v>
@@ -2094,19 +2091,19 @@
         <v>36</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G22" s="3"/>
     </row>
     <row r="23" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B23" s="5">
         <v>2022</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>37</v>
@@ -2115,19 +2112,19 @@
         <v>38</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G23" s="3"/>
     </row>
     <row r="24" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B24" s="5">
         <v>2022</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>37</v>
@@ -2136,19 +2133,19 @@
         <v>39</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G24" s="3"/>
     </row>
     <row r="25" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B25" s="5">
         <v>2023</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>40</v>
@@ -2157,19 +2154,19 @@
         <v>41</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G25" s="3"/>
     </row>
     <row r="26" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B26" s="5">
         <v>2025</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>42</v>
@@ -2178,19 +2175,19 @@
         <v>43</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G26" s="3"/>
     </row>
     <row r="27" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B27" s="5">
         <v>2015</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>44</v>
@@ -2199,19 +2196,19 @@
         <v>45</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G27" s="3"/>
     </row>
     <row r="28" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B28" s="5">
         <v>2015</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>44</v>
@@ -2220,19 +2217,19 @@
         <v>46</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G28" s="3"/>
     </row>
     <row r="29" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B29" s="5">
         <v>2015</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>44</v>
@@ -2241,19 +2238,19 @@
         <v>47</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G29" s="3"/>
     </row>
     <row r="30" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B30" s="5">
         <v>2025</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>48</v>
@@ -2262,19 +2259,19 @@
         <v>49</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B31" s="5">
         <v>2025</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>50</v>
@@ -2283,19 +2280,19 @@
         <v>51</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G31" s="3"/>
     </row>
     <row r="32" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B32" s="5">
         <v>2025</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>50</v>
@@ -2304,19 +2301,19 @@
         <v>52</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G32" s="3"/>
     </row>
     <row r="33" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B33" s="5">
         <v>2025</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>53</v>
@@ -2328,18 +2325,18 @@
         <v>172</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B34" s="5">
         <v>2025</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>53</v>
@@ -2354,13 +2351,13 @@
     </row>
     <row r="35" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B35" s="5">
         <v>2015</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>56</v>
@@ -2369,19 +2366,19 @@
         <v>57</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>173</v>
+        <v>210</v>
       </c>
       <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B36" s="5">
         <v>2015</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>56</v>
@@ -2390,19 +2387,19 @@
         <v>58</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G36" s="3"/>
     </row>
     <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B37" s="5">
         <v>2015</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>59</v>
@@ -2411,19 +2408,19 @@
         <v>60</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G37" s="3"/>
     </row>
     <row r="38" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B38" s="5">
         <v>2025</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>61</v>
@@ -2432,19 +2429,19 @@
         <v>62</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G38" s="3"/>
     </row>
     <row r="39" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B39" s="5">
         <v>2025</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>61</v>
@@ -2453,19 +2450,19 @@
         <v>63</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G39" s="3"/>
     </row>
     <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B40" s="5">
         <v>2025</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>64</v>
@@ -2480,13 +2477,13 @@
     </row>
     <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B41" s="5">
         <v>2025</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>64</v>
@@ -2495,19 +2492,19 @@
         <v>66</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G41" s="3"/>
     </row>
     <row r="42" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B42" s="5">
         <v>2025</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>67</v>
@@ -2516,19 +2513,19 @@
         <v>68</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G42" s="3"/>
     </row>
     <row r="43" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B43" s="5">
         <v>2025</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>67</v>
@@ -2537,19 +2534,19 @@
         <v>69</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G43" s="3"/>
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B44" s="5">
         <v>2025</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>67</v>
@@ -2558,21 +2555,21 @@
         <v>70</v>
       </c>
       <c r="F44" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G44" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="G44" s="3" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B45" s="5">
         <v>2025</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>71</v>
@@ -2581,19 +2578,19 @@
         <v>72</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G45" s="3"/>
     </row>
     <row r="46" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B46" s="5">
         <v>2025</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>71</v>
@@ -2602,19 +2599,19 @@
         <v>73</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G46" s="3"/>
     </row>
     <row r="47" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B47" s="5">
         <v>2025</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>74</v>
@@ -2623,19 +2620,19 @@
         <v>75</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G47" s="3"/>
     </row>
     <row r="48" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B48" s="5">
         <v>2025</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>74</v>
@@ -2644,19 +2641,19 @@
         <v>76</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G48" s="3"/>
     </row>
     <row r="49" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B49" s="5">
         <v>2025</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>77</v>
@@ -2665,19 +2662,19 @@
         <v>78</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G49" s="3"/>
     </row>
     <row r="50" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B50" s="5">
         <v>2025</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>77</v>
@@ -2686,19 +2683,19 @@
         <v>79</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G50" s="3"/>
     </row>
     <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B51" s="5">
         <v>2025</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>80</v>
@@ -2707,21 +2704,21 @@
         <v>81</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B52" s="5">
         <v>2022</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>82</v>
@@ -2730,19 +2727,19 @@
         <v>83</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G52" s="3"/>
     </row>
     <row r="53" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B53" s="5">
         <v>2022</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>82</v>
@@ -2751,19 +2748,19 @@
         <v>84</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G53" s="3"/>
     </row>
     <row r="54" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B54" s="5">
         <v>2025</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>85</v>
@@ -2772,19 +2769,19 @@
         <v>86</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G54" s="3"/>
     </row>
     <row r="55" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A55" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B55" s="5">
         <v>2025</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>85</v>
@@ -2793,19 +2790,19 @@
         <v>87</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G55" s="3"/>
     </row>
     <row r="56" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A56" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B56" s="5">
         <v>2015</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>88</v>
@@ -2814,19 +2811,19 @@
         <v>89</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G56" s="3"/>
     </row>
     <row r="57" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A57" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B57" s="5">
         <v>2025</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>90</v>
@@ -2835,19 +2832,19 @@
         <v>91</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G57" s="3"/>
     </row>
     <row r="58" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B58" s="5">
         <v>2025</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>92</v>
@@ -2856,19 +2853,19 @@
         <v>93</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G58" s="3"/>
     </row>
     <row r="59" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A59" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B59" s="5">
         <v>2025</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>92</v>
@@ -2877,19 +2874,19 @@
         <v>94</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G59" s="3"/>
     </row>
     <row r="60" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A60" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B60" s="5">
         <v>2015</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>95</v>
@@ -2898,19 +2895,19 @@
         <v>96</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G60" s="3"/>
     </row>
     <row r="61" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A61" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B61" s="5">
         <v>2015</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>95</v>
@@ -2919,19 +2916,19 @@
         <v>97</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G61" s="3"/>
     </row>
     <row r="62" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B62" s="5">
         <v>2025</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>98</v>
@@ -2940,19 +2937,19 @@
         <v>99</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G62" s="3"/>
     </row>
     <row r="63" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A63" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B63" s="5">
         <v>2025</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>100</v>
@@ -2964,18 +2961,18 @@
         <v>172</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A64" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B64" s="5">
         <v>2025</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>102</v>
@@ -2984,21 +2981,21 @@
         <v>103</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B65" s="5">
         <v>2025</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>102</v>
@@ -3007,21 +3004,21 @@
         <v>104</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B66" s="5">
         <v>2015</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>105</v>
@@ -3030,19 +3027,19 @@
         <v>106</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G66" s="3"/>
     </row>
     <row r="67" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B67" s="5">
         <v>2015</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>105</v>
@@ -3051,19 +3048,19 @@
         <v>107</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G67" s="3"/>
     </row>
     <row r="68" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B68" s="5">
         <v>2023</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>108</v>
@@ -3072,19 +3069,19 @@
         <v>109</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G68" s="3"/>
     </row>
     <row r="69" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B69" s="5">
         <v>2023</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>108</v>
@@ -3093,19 +3090,19 @@
         <v>110</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G69" s="3"/>
     </row>
     <row r="70" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B70" s="5">
         <v>2025</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>111</v>
@@ -3120,13 +3117,13 @@
     </row>
     <row r="71" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A71" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B71" s="5">
         <v>2025</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>113</v>
@@ -3141,13 +3138,13 @@
     </row>
     <row r="72" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B72" s="5">
         <v>2025</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>113</v>
@@ -3156,61 +3153,61 @@
         <v>115</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G72" s="3"/>
     </row>
     <row r="73" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B73" s="5">
         <v>2015</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>177</v>
+        <v>224</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>116</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G73" s="3"/>
     </row>
     <row r="74" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B74" s="5">
         <v>2015</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>177</v>
+        <v>224</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>117</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G74" s="3"/>
     </row>
     <row r="75" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B75" s="5">
         <v>2015</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>118</v>
@@ -3219,19 +3216,19 @@
         <v>119</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G75" s="3"/>
     </row>
     <row r="76" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B76" s="5">
         <v>2015</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>118</v>
@@ -3246,13 +3243,13 @@
     </row>
     <row r="77" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B77" s="5">
         <v>2025</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>121</v>
@@ -3261,19 +3258,19 @@
         <v>122</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G77" s="3"/>
     </row>
     <row r="78" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A78" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B78" s="5">
         <v>2025</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>121</v>
@@ -3282,19 +3279,19 @@
         <v>123</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G78" s="3"/>
     </row>
     <row r="79" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A79" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B79" s="5">
         <v>2025</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>124</v>
@@ -3303,19 +3300,19 @@
         <v>125</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G79" s="3"/>
     </row>
     <row r="80" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B80" s="5">
         <v>2015</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>126</v>
@@ -3324,19 +3321,19 @@
         <v>127</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G80" s="3"/>
     </row>
     <row r="81" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B81" s="5">
         <v>2017</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>128</v>
@@ -3345,19 +3342,19 @@
         <v>129</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G81" s="3"/>
     </row>
     <row r="82" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B82" s="5">
         <v>2017</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>128</v>
@@ -3366,19 +3363,19 @@
         <v>130</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G82" s="3"/>
     </row>
     <row r="83" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B83" s="5">
         <v>2020</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>2</v>
@@ -3393,13 +3390,13 @@
     </row>
     <row r="84" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B84" s="5">
         <v>2020</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>8</v>
@@ -3414,13 +3411,13 @@
     </row>
     <row r="85" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B85" s="5">
         <v>2020</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>8</v>
@@ -3429,19 +3426,19 @@
         <v>133</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G85" s="3"/>
     </row>
     <row r="86" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B86" s="5">
         <v>2020</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>11</v>
@@ -3456,13 +3453,13 @@
     </row>
     <row r="87" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B87" s="5">
         <v>2020</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>11</v>
@@ -3477,13 +3474,13 @@
     </row>
     <row r="88" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B88" s="5">
         <v>2020</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>17</v>
@@ -3492,19 +3489,19 @@
         <v>136</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G88" s="3"/>
     </row>
     <row r="89" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A89" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B89" s="5">
         <v>2020</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
@@ -3513,19 +3510,19 @@
         <v>137</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G89" s="3"/>
     </row>
     <row r="90" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A90" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B90" s="5">
         <v>2020</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>19</v>
@@ -3534,19 +3531,19 @@
         <v>138</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G90" s="3"/>
     </row>
     <row r="91" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A91" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B91" s="5">
         <v>2020</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>24</v>
@@ -3555,19 +3552,19 @@
         <v>139</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G91" s="3"/>
     </row>
     <row r="92" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A92" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B92" s="5">
         <v>2020</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>26</v>
@@ -3576,19 +3573,19 @@
         <v>140</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G92" s="3"/>
     </row>
     <row r="93" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B93" s="5">
         <v>2020</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>44</v>
@@ -3597,19 +3594,19 @@
         <v>141</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G93" s="3"/>
     </row>
     <row r="94" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B94" s="5">
         <v>2020</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>44</v>
@@ -3618,19 +3615,19 @@
         <v>142</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G94" s="3"/>
     </row>
     <row r="95" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A95" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B95" s="5">
         <v>2020</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>48</v>
@@ -3645,13 +3642,13 @@
     </row>
     <row r="96" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A96" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B96" s="5">
         <v>2020</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>48</v>
@@ -3660,19 +3657,19 @@
         <v>144</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G96" s="3"/>
     </row>
     <row r="97" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A97" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B97" s="5">
         <v>2020</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>50</v>
@@ -3681,19 +3678,19 @@
         <v>145</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G97" s="3"/>
     </row>
     <row r="98" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A98" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B98" s="5">
         <v>2020</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>53</v>
@@ -3702,19 +3699,19 @@
         <v>146</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G98" s="3"/>
     </row>
     <row r="99" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A99" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B99" s="5">
         <v>2020</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>56</v>
@@ -3723,19 +3720,19 @@
         <v>147</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="G99" s="3"/>
     </row>
     <row r="100" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A100" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B100" s="5">
         <v>2020</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>56</v>
@@ -3744,19 +3741,19 @@
         <v>148</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G100" s="3"/>
     </row>
     <row r="101" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A101" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B101" s="5">
         <v>2022</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>59</v>
@@ -3765,19 +3762,19 @@
         <v>149</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G101" s="3"/>
     </row>
     <row r="102" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B102" s="5">
         <v>2022</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>59</v>
@@ -3786,19 +3783,19 @@
         <v>150</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G102" s="3"/>
     </row>
     <row r="103" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A103" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B103" s="5">
         <v>2020</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>64</v>
@@ -3807,19 +3804,19 @@
         <v>151</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G103" s="3"/>
     </row>
     <row r="104" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A104" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B104" s="5">
         <v>2020</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>77</v>
@@ -3828,19 +3825,19 @@
         <v>152</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G104" s="3"/>
     </row>
     <row r="105" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A105" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B105" s="5">
         <v>2020</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>153</v>
@@ -3849,19 +3846,19 @@
         <v>154</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G105" s="3"/>
     </row>
     <row r="106" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A106" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B106" s="5">
         <v>2020</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>153</v>
@@ -3870,19 +3867,19 @@
         <v>155</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G106" s="3"/>
     </row>
     <row r="107" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A107" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B107" s="5">
         <v>2020</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>85</v>
@@ -3891,19 +3888,19 @@
         <v>156</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G107" s="3"/>
     </row>
     <row r="108" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A108" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B108" s="5">
         <v>2020</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>85</v>
@@ -3912,21 +3909,21 @@
         <v>157</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A109" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B109" s="5">
         <v>2020</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>88</v>
@@ -3941,13 +3938,13 @@
     </row>
     <row r="110" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A110" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B110" s="5">
         <v>2020</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>90</v>
@@ -3956,19 +3953,21 @@
         <v>159</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="G110" s="3"/>
+        <v>196</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="111" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A111" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B111" s="5">
         <v>2020</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>92</v>
@@ -3977,19 +3976,19 @@
         <v>160</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G111" s="3"/>
     </row>
     <row r="112" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A112" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B112" s="5">
         <v>2020</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>161</v>
@@ -4004,13 +4003,13 @@
     </row>
     <row r="113" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A113" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B113" s="5">
         <v>2020</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>161</v>
@@ -4019,19 +4018,19 @@
         <v>163</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G113" s="3"/>
     </row>
     <row r="114" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A114" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B114" s="5">
         <v>2020</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>98</v>
@@ -4040,21 +4039,21 @@
         <v>164</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A115" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B115" s="5">
         <v>2020</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>98</v>
@@ -4063,19 +4062,19 @@
         <v>165</v>
       </c>
       <c r="F115" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G115" s="5"/>
     </row>
     <row r="116" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A116" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B116" s="5">
         <v>2020</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>105</v>
@@ -4084,19 +4083,19 @@
         <v>166</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G116" s="3"/>
     </row>
     <row r="117" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A117" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B117" s="5">
         <v>2020</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>105</v>
@@ -4105,19 +4104,19 @@
         <v>167</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G117" s="3"/>
     </row>
     <row r="118" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A118" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B118" s="5">
         <v>2020</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>113</v>
@@ -4126,19 +4125,19 @@
         <v>168</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G118" s="3"/>
     </row>
     <row r="119" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A119" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B119" s="5">
         <v>2025</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>121</v>
@@ -4147,19 +4146,19 @@
         <v>169</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G119" s="3"/>
     </row>
     <row r="120" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A120" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B120" s="5">
         <v>2025</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>121</v>
@@ -4168,19 +4167,19 @@
         <v>170</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G120" s="3"/>
     </row>
     <row r="121" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A121" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B121" s="5">
         <v>2020</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>124</v>
@@ -4189,7 +4188,7 @@
         <v>171</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G121" s="3"/>
     </row>
@@ -4209,16 +4208,16 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>195</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="102" x14ac:dyDescent="0.2">
@@ -4226,79 +4225,79 @@
         <v>172</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="102" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="102" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="85" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>